<commit_message>
Informe y ajustes modelo relacional modulo 9
</commit_message>
<xml_diff>
--- a/Nomenclatura.xlsx
+++ b/Nomenclatura.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samue\Documents\USCO\8Semestre\IntegradorIII\documentacionDB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFEE68A9-1703-45D4-9925-631F52268D5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A71C9E7-1D20-460A-A5FF-77EAE02524AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -446,62 +446,6 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="12"/>
-        <name val="Roboto"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Roboto"/>
-        <scheme val="none"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Roboto"/>
-        <scheme val="none"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
         <color auto="1"/>
         <name val="Roboto"/>
         <scheme val="none"/>
@@ -626,6 +570,28 @@
       </border>
     </dxf>
     <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Roboto"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
@@ -642,10 +608,44 @@
       </border>
     </dxf>
     <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Roboto"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
       <border>
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Roboto"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
       </border>
     </dxf>
     <dxf>
@@ -709,13 +709,13 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="VERSION_1.0.0" displayName="VERSION_1.0.0" ref="A1:E15" headerRowDxfId="2" dataDxfId="0" totalsRowDxfId="1" headerRowBorderDxfId="9" tableBorderDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="VERSION_1.0.0" displayName="VERSION_1.0.0" ref="A1:E15" headerRowDxfId="9" dataDxfId="7" totalsRowDxfId="5" headerRowBorderDxfId="8" tableBorderDxfId="6">
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Categoría" dataDxfId="7"/>
-    <tableColumn id="5" xr3:uid="{6A73C46B-9990-4E71-BFB1-AB23671C894F}" name="Tipo" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Elemento" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Convención / Regla" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Comentarios" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Categoría" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{6A73C46B-9990-4E71-BFB1-AB23671C894F}" name="Tipo" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Elemento" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Convención / Regla" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Comentarios" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="Modulo 1-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>

</xml_diff>